<commit_message>
Update Prom price file
</commit_message>
<xml_diff>
--- a/prom.xlsx
+++ b/prom.xlsx
@@ -1026,7 +1026,7 @@
         </is>
       </c>
       <c r="Q2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="R2" t="n">
         <v>143279712</v>
@@ -1510,11 +1510,11 @@
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>+</t>
         </is>
       </c>
       <c r="Q4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="R4" t="n">
         <v>143279712</v>
@@ -24042,7 +24042,7 @@
         </is>
       </c>
       <c r="Q81" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="R81" t="n">
         <v>143878720</v>
@@ -36926,7 +36926,7 @@
         </is>
       </c>
       <c r="Q128" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="R128" t="n">
         <v>143878719</v>

</xml_diff>